<commit_message>
feat: adicionar linha de 720 dias (504 DUs) em todos os modelos de mailer
- 720 dias adicionado nos 7 modelos de tabela (modelo 1-5, fapes, funcef)
- Logica de filtragem: remove 720 quando fundo tem < 505 DUs
- Limpeza de linhas sobressalentes no template (evita Acumulado duplicado)
- Garantia de linha vazia antes do Patrimonio Liquido
- Validacao de labels duplicados antes de gerar email
- Send() temporariamente desativado (Display apenas) ate 16/04/2026
- Backup do original em versoes/mailer_v_oficial_IPCA_ANTES_720.py

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/3M HARPIA - template.xlsx
+++ b/templates/3M HARPIA - template.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="20355" yWindow="-11640" windowWidth="20730" windowHeight="11040" tabRatio="711" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Email" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="DataAnálise">Email!$A$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Email'!$B$7:$G$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Email'!$B$7:$G$43</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -1251,7 +1251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="13.42578125" customWidth="1" style="57" min="1" max="1"/>
@@ -1259,8 +1259,8 @@
     <col width="5.42578125" customWidth="1" style="57" min="8" max="8"/>
     <col width="23.140625" bestFit="1" customWidth="1" style="57" min="9" max="9"/>
     <col width="23.42578125" bestFit="1" customWidth="1" style="57" min="10" max="10"/>
-    <col width="9.140625" customWidth="1" style="57" min="11" max="16"/>
-    <col width="9.140625" customWidth="1" style="57" min="17" max="16384"/>
+    <col width="9.140625" customWidth="1" style="57" min="11" max="17"/>
+    <col width="9.140625" customWidth="1" style="57" min="18" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1417,23 +1417,23 @@
       <c r="A17" s="4" t="n"/>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="C17" s="10" t="n">
-        <v>3.4655033</v>
+        <v>3.4979167</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>0.000960522593611346</v>
+        <v>0.0004694710396517809</v>
       </c>
       <c r="E17" s="11" t="n">
-        <v>0.0004925342348984785</v>
+        <v>0.0004308998088589089</v>
       </c>
       <c r="F17" s="11" t="n">
         <v>0.0005426623598601132</v>
       </c>
       <c r="G17" s="40" t="n">
-        <v>1.770018826916516</v>
+        <v>0.8651254893978653</v>
       </c>
       <c r="H17" s="4" t="n"/>
     </row>
@@ -1441,23 +1441,23 @@
       <c r="A18" s="4" t="n"/>
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="C18" s="28" t="n">
-        <v>3.4621778</v>
+        <v>3.4962753</v>
       </c>
       <c r="D18" s="29" t="n">
-        <v>-0.0001895557113302804</v>
+        <v>4.22467417953154e-05</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>0.0004925342348984785</v>
+        <v>0.0004308998088589089</v>
       </c>
       <c r="F18" s="29" t="n">
         <v>0.0005426623598601132</v>
       </c>
       <c r="G18" s="30" t="n">
-        <v>-0.3493069085888761</v>
+        <v>0.07785087914740522</v>
       </c>
       <c r="H18" s="4" t="n"/>
     </row>
@@ -1465,23 +1465,23 @@
       <c r="A19" s="4" t="n"/>
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C19" s="28" t="n">
-        <v>3.4628342</v>
+        <v>3.4961276</v>
       </c>
       <c r="D19" s="29" t="n">
-        <v>0.0006577551943935944</v>
+        <v>0.0009981270622823057</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0004925342348984785</v>
+        <v>0.0004308998088589089</v>
       </c>
       <c r="F19" s="29" t="n">
         <v>0.0005426623598601132</v>
       </c>
       <c r="G19" s="30" t="n">
-        <v>1.212089216143809</v>
+        <v>1.839315080816738</v>
       </c>
       <c r="H19" s="4" t="n"/>
     </row>
@@ -1489,23 +1489,23 @@
       <c r="A20" s="4" t="n"/>
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="C20" s="28" t="n">
-        <v>3.460558</v>
+        <v>3.4926415</v>
       </c>
       <c r="D20" s="29" t="n">
-        <v>0.0003950345044498871</v>
+        <v>-0.0001048380168185981</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.0004925342348984785</v>
+        <v>0.0004308998088589089</v>
       </c>
       <c r="F20" s="29" t="n">
         <v>0.0005426623598601132</v>
       </c>
       <c r="G20" s="30" t="n">
-        <v>0.7279563383605941</v>
+        <v>-0.1931919819270735</v>
       </c>
       <c r="H20" s="4" t="n"/>
     </row>
@@ -1513,23 +1513,23 @@
       <c r="A21" s="4" t="n"/>
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C21" s="28" t="n">
-        <v>3.4591915</v>
+        <v>3.4930077</v>
       </c>
       <c r="D21" s="29" t="n">
-        <v>-0.0001818013391157169</v>
+        <v>0.002246772352155535</v>
       </c>
       <c r="E21" s="29" t="n">
-        <v>0.0004925342348984785</v>
+        <v>0.0004308998088589089</v>
       </c>
       <c r="F21" s="29" t="n">
-        <v>0.0005513106415402369</v>
+        <v>0.0005426623598601132</v>
       </c>
       <c r="G21" s="30" t="n">
-        <v>-0.3297620713574569</v>
+        <v>4.140276750970354</v>
       </c>
       <c r="H21" s="4" t="n"/>
     </row>
@@ -1577,21 +1577,21 @@
       <c r="A24" s="4" t="n"/>
       <c r="B24" s="45" t="inlineStr">
         <is>
-          <t>Mar-26</t>
+          <t>Apr-26</t>
         </is>
       </c>
       <c r="C24" s="47" t="inlineStr"/>
       <c r="D24" s="11" t="n">
-        <v>0.01042422673973875</v>
+        <v>0.007225648365121407</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>0.008902830173136644</v>
+        <v>0.003020200631021153</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>0.00993531358511679</v>
+        <v>0.003804826246388782</v>
       </c>
       <c r="G24" s="16" t="n">
-        <v>1.049209634948449</v>
+        <v>1.899074464170178</v>
       </c>
       <c r="H24" s="17" t="n"/>
     </row>
@@ -1604,16 +1604,16 @@
       </c>
       <c r="C25" s="43" t="inlineStr"/>
       <c r="D25" s="29" t="n">
-        <v>0.01452925711645259</v>
+        <v>0.01276977327343465</v>
       </c>
       <c r="E25" s="31" t="n">
-        <v>0.010609435333087</v>
+        <v>0.0121671107114012</v>
       </c>
       <c r="F25" s="31" t="n">
-        <v>0.01160659890087934</v>
+        <v>0.0115104208368324</v>
       </c>
       <c r="G25" s="32" t="n">
-        <v>1.251810047071741</v>
+        <v>1.109409764808287</v>
       </c>
       <c r="H25" s="17" t="n"/>
     </row>
@@ -1626,16 +1626,16 @@
       </c>
       <c r="C26" s="43" t="inlineStr"/>
       <c r="D26" s="29" t="n">
-        <v>0.03483383848186694</v>
+        <v>0.04164468355924233</v>
       </c>
       <c r="E26" s="31" t="n">
-        <v>0.0299218930353895</v>
+        <v>0.03420344006821918</v>
       </c>
       <c r="F26" s="31" t="n">
-        <v>0.03529708637135154</v>
+        <v>0.03519865594435645</v>
       </c>
       <c r="G26" s="32" t="n">
-        <v>0.9868757470627778</v>
+        <v>1.183132777145697</v>
       </c>
       <c r="H26" s="17" t="n"/>
     </row>
@@ -1648,16 +1648,16 @@
       </c>
       <c r="C27" s="43" t="inlineStr"/>
       <c r="D27" s="29" t="n">
-        <v>0.0709049659041241</v>
+        <v>0.07453166598582706</v>
       </c>
       <c r="E27" s="31" t="n">
-        <v>0.05159954897003649</v>
+        <v>0.05631847919317901</v>
       </c>
       <c r="F27" s="31" t="n">
-        <v>0.07187711571831934</v>
+        <v>0.07177520746070365</v>
       </c>
       <c r="G27" s="32" t="n">
-        <v>0.9864748354955557</v>
+        <v>1.038404048175445</v>
       </c>
       <c r="H27" s="17" t="n"/>
     </row>
@@ -1670,16 +1670,16 @@
       </c>
       <c r="C28" s="43" t="inlineStr"/>
       <c r="D28" s="29" t="n">
-        <v>0.1486280909186244</v>
+        <v>0.1520928554939127</v>
       </c>
       <c r="E28" s="31" t="n">
-        <v>0.09976390624150056</v>
+        <v>0.1034873929584561</v>
       </c>
       <c r="F28" s="31" t="n">
-        <v>0.1477970366518437</v>
+        <v>0.148016036262707</v>
       </c>
       <c r="G28" s="32" t="n">
-        <v>1.005622942689564</v>
+        <v>1.02754309150645</v>
       </c>
       <c r="H28" s="17" t="n"/>
     </row>
@@ -1687,65 +1687,65 @@
       <c r="A29" s="27" t="n"/>
       <c r="B29" s="48" t="inlineStr">
         <is>
-          <t>Ano 2026</t>
+          <t>Últimos 720 dias</t>
         </is>
       </c>
       <c r="C29" s="43" t="inlineStr"/>
       <c r="D29" s="29" t="n">
-        <v>0.03189672979121294</v>
+        <v>0.2431223100136561</v>
       </c>
       <c r="E29" s="31" t="n">
-        <v>0.02752636552488252</v>
+        <v>0.2331517508618997</v>
       </c>
       <c r="F29" s="31" t="n">
-        <v>0.03187906296972676</v>
+        <v>0.2779304689804314</v>
       </c>
       <c r="G29" s="32" t="n">
-        <v>1.000554182583816</v>
+        <v>0.8747594709768002</v>
       </c>
       <c r="H29" s="17" t="n"/>
     </row>
-    <row r="30" ht="15.95" customHeight="1">
+    <row r="30" ht="15.95" customFormat="1" customHeight="1" s="26">
       <c r="A30" s="27" t="n"/>
       <c r="B30" s="48" t="inlineStr">
         <is>
-          <t>Ano 2025</t>
+          <t>Ano 2026</t>
         </is>
       </c>
       <c r="C30" s="43" t="inlineStr"/>
       <c r="D30" s="29" t="n">
-        <v>0.1479691460436279</v>
+        <v>0.04154822297011562</v>
       </c>
       <c r="E30" s="31" t="n">
-        <v>0.1042657310150845</v>
+        <v>0.03621228344143779</v>
       </c>
       <c r="F30" s="31" t="n">
-        <v>0.143132751155109</v>
+        <v>0.0380553842733744</v>
       </c>
       <c r="G30" s="32" t="n">
-        <v>1.033789575408061</v>
-      </c>
-      <c r="H30" s="55" t="n"/>
+        <v>1.091783035789367</v>
+      </c>
+      <c r="H30" s="17" t="n"/>
     </row>
     <row r="31" ht="15.95" customHeight="1">
       <c r="A31" s="27" t="n"/>
       <c r="B31" s="48" t="inlineStr">
         <is>
-          <t>Ano 2024</t>
+          <t>Ano 2025</t>
         </is>
       </c>
       <c r="C31" s="43" t="inlineStr"/>
       <c r="D31" s="29" t="n">
-        <v>0.07456125884066322</v>
+        <v>0.1479691460436279</v>
       </c>
       <c r="E31" s="31" t="n">
-        <v>0.1113897041597771</v>
+        <v>0.1042657310150845</v>
       </c>
       <c r="F31" s="31" t="n">
-        <v>0.1092049264357533</v>
+        <v>0.143132751155109</v>
       </c>
       <c r="G31" s="32" t="n">
-        <v>0.6827646084678112</v>
+        <v>1.033789575408061</v>
       </c>
       <c r="H31" s="55" t="n"/>
     </row>
@@ -1753,185 +1753,207 @@
       <c r="A32" s="27" t="n"/>
       <c r="B32" s="48" t="inlineStr">
         <is>
-          <t>Acumulado²</t>
+          <t>Ano 2024</t>
         </is>
       </c>
       <c r="C32" s="43" t="inlineStr"/>
       <c r="D32" s="29" t="n">
-        <v>2.4655033</v>
+        <v>0.07456125884066322</v>
       </c>
       <c r="E32" s="31" t="n">
-        <v>3.551354177874543</v>
+        <v>0.1113897041597771</v>
       </c>
       <c r="F32" s="31" t="n">
-        <v>2.450522326552379</v>
+        <v>0.1092049264357533</v>
       </c>
       <c r="G32" s="32" t="n">
-        <v>1.006113379700848</v>
+        <v>0.6827646084678112</v>
       </c>
       <c r="H32" s="55" t="n"/>
     </row>
     <row r="33" ht="15.95" customHeight="1">
-      <c r="A33" s="4" t="n"/>
-      <c r="B33" s="19" t="n"/>
-      <c r="C33" s="13" t="n"/>
-      <c r="D33" s="13" t="n"/>
-      <c r="E33" s="13" t="n"/>
-      <c r="F33" s="13" t="n"/>
-      <c r="G33" s="13" t="n"/>
-      <c r="H33" s="4" t="n"/>
-    </row>
-    <row r="34" ht="26.1" customHeight="1">
-      <c r="B34" s="56" t="inlineStr">
+      <c r="A33" s="27" t="n"/>
+      <c r="B33" s="48" t="inlineStr">
+        <is>
+          <t>Acumulado²</t>
+        </is>
+      </c>
+      <c r="C33" s="43" t="inlineStr"/>
+      <c r="D33" s="29" t="n">
+        <v>2.4979167</v>
+      </c>
+      <c r="E33" s="31" t="n">
+        <v>3.589827826945334</v>
+      </c>
+      <c r="F33" s="31" t="n">
+        <v>2.471175458609215</v>
+      </c>
+      <c r="G33" s="32" t="n">
+        <v>1.010821263742169</v>
+      </c>
+      <c r="H33" s="55" t="n"/>
+    </row>
+    <row r="34" ht="15.95" customHeight="1">
+      <c r="A34" s="4" t="n"/>
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="13" t="n"/>
+      <c r="D34" s="13" t="n"/>
+      <c r="E34" s="13" t="n"/>
+      <c r="F34" s="13" t="n"/>
+      <c r="G34" s="13" t="n"/>
+      <c r="H34" s="4" t="n"/>
+    </row>
+    <row r="35" ht="26.1" customHeight="1">
+      <c r="B35" s="56" t="inlineStr">
         <is>
           <t>Patrimônio Líquido (R$)</t>
         </is>
       </c>
-      <c r="H34" s="4" t="n"/>
-    </row>
-    <row r="35" ht="15.95" customHeight="1">
-      <c r="B35" s="33" t="inlineStr">
+      <c r="H35" s="4" t="n"/>
+    </row>
+    <row r="36" ht="15.95" customHeight="1">
+      <c r="B36" s="33" t="inlineStr">
         <is>
           <t>Hoje¹</t>
-        </is>
-      </c>
-      <c r="C35" s="34" t="n"/>
-      <c r="D35" s="34" t="n"/>
-      <c r="E35" s="44" t="n">
-        <v>71498981.31999999</v>
-      </c>
-      <c r="F35" s="44" t="n"/>
-      <c r="G35" s="44" t="n"/>
-      <c r="H35" s="4" t="n"/>
-    </row>
-    <row r="36" ht="15.95" customHeight="1">
-      <c r="B36" s="35" t="inlineStr">
-        <is>
-          <t>Últimos 12 Meses (Média Diária)¹</t>
         </is>
       </c>
       <c r="C36" s="34" t="n"/>
       <c r="D36" s="34" t="n"/>
       <c r="E36" s="44" t="n">
-        <v>72707188.59432539</v>
+        <v>72167723.03</v>
       </c>
       <c r="F36" s="44" t="n"/>
       <c r="G36" s="44" t="n"/>
       <c r="H36" s="4" t="n"/>
     </row>
     <row r="37" ht="15.95" customHeight="1">
-      <c r="B37" s="33" t="n"/>
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>Últimos 12 Meses (Média Diária)¹</t>
+        </is>
+      </c>
       <c r="C37" s="34" t="n"/>
       <c r="D37" s="34" t="n"/>
-      <c r="E37" s="34" t="n"/>
-      <c r="F37" s="34" t="n"/>
-      <c r="G37" s="34" t="n"/>
+      <c r="E37" s="44" t="n">
+        <v>70529141.235</v>
+      </c>
+      <c r="F37" s="44" t="n"/>
+      <c r="G37" s="44" t="n"/>
       <c r="H37" s="4" t="n"/>
     </row>
     <row r="38" ht="15.95" customHeight="1">
-      <c r="A38" s="4" t="n"/>
-      <c r="B38" s="36" t="inlineStr">
-        <is>
-          <t>¹Data de Referência:</t>
-        </is>
-      </c>
-      <c r="C38" s="41" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-      <c r="D38" s="37" t="n"/>
-      <c r="E38" s="37" t="n"/>
-      <c r="F38" s="37" t="n"/>
-      <c r="G38" s="37" t="n"/>
+      <c r="B38" s="33" t="n"/>
+      <c r="C38" s="34" t="n"/>
+      <c r="D38" s="34" t="n"/>
+      <c r="E38" s="34" t="n"/>
+      <c r="F38" s="34" t="n"/>
+      <c r="G38" s="34" t="n"/>
       <c r="H38" s="4" t="n"/>
     </row>
     <row r="39" ht="15.95" customHeight="1">
       <c r="A39" s="4" t="n"/>
-      <c r="B39" s="38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">² Cota Inicial em: </t>
+      <c r="B39" s="36" t="inlineStr">
+        <is>
+          <t>¹Data de Referência:</t>
         </is>
       </c>
       <c r="C39" s="41" t="inlineStr">
         <is>
-          <t>2012-11-07</t>
-        </is>
-      </c>
-      <c r="D39" s="39" t="n"/>
-      <c r="E39" s="39" t="n"/>
-      <c r="F39" s="39" t="n"/>
-      <c r="G39" s="39" t="n"/>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="D39" s="37" t="n"/>
+      <c r="E39" s="37" t="n"/>
+      <c r="F39" s="37" t="n"/>
+      <c r="G39" s="37" t="n"/>
       <c r="H39" s="4" t="n"/>
     </row>
     <row r="40" ht="15.95" customHeight="1">
       <c r="A40" s="4" t="n"/>
-      <c r="B40" s="21" t="n"/>
-      <c r="C40" s="20" t="n"/>
-      <c r="D40" s="22" t="n"/>
-      <c r="E40" s="22" t="n"/>
-      <c r="F40" s="22" t="n"/>
-      <c r="G40" s="22" t="n"/>
+      <c r="B40" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">² Cota Inicial em: </t>
+        </is>
+      </c>
+      <c r="C40" s="41" t="inlineStr">
+        <is>
+          <t>2012-11-07</t>
+        </is>
+      </c>
+      <c r="D40" s="39" t="n"/>
+      <c r="E40" s="39" t="n"/>
+      <c r="F40" s="39" t="n"/>
+      <c r="G40" s="39" t="n"/>
       <c r="H40" s="4" t="n"/>
     </row>
-    <row r="41" ht="40.5" customHeight="1">
+    <row r="41" ht="15.95" customHeight="1">
       <c r="A41" s="4" t="n"/>
-      <c r="B41" s="50" t="inlineStr">
+      <c r="B41" s="21" t="n"/>
+      <c r="C41" s="20" t="n"/>
+      <c r="D41" s="22" t="n"/>
+      <c r="E41" s="22" t="n"/>
+      <c r="F41" s="22" t="n"/>
+      <c r="G41" s="22" t="n"/>
+      <c r="H41" s="4" t="n"/>
+    </row>
+    <row r="42" ht="40.5" customHeight="1">
+      <c r="A42" s="4" t="n"/>
+      <c r="B42" s="50" t="inlineStr">
         <is>
           <t>As informações contidas neste material são de caráter exclusivamente informativo. Fundos de investimento não contam com garantia do administrador do fundo, do gestor da carteira, de qualquer mecanismo de seguro ou, ainda, do Fundo Garantidor de Créditos – FGC. Rentabilidade passada não representa garantia de rentabilidade futura. "A rentabilidade divulgada não é líquida de impostos.“ Leia o prospecto e o regulamento antes de investir.</t>
         </is>
       </c>
-      <c r="C41" s="50" t="n"/>
-      <c r="D41" s="50" t="n"/>
-      <c r="E41" s="50" t="n"/>
-      <c r="F41" s="50" t="n"/>
-      <c r="G41" s="50" t="n"/>
-      <c r="H41" s="4" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="n"/>
-      <c r="B42" s="49" t="n"/>
-      <c r="C42" s="49" t="n"/>
-      <c r="D42" s="49" t="n"/>
-      <c r="E42" s="49" t="n"/>
-      <c r="F42" s="49" t="n"/>
-      <c r="G42" s="49" t="n"/>
+      <c r="C42" s="50" t="n"/>
+      <c r="D42" s="50" t="n"/>
+      <c r="E42" s="50" t="n"/>
+      <c r="F42" s="50" t="n"/>
+      <c r="G42" s="50" t="n"/>
       <c r="H42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n"/>
-      <c r="B43" s="23" t="n"/>
-      <c r="C43" s="23" t="n"/>
-      <c r="D43" s="23" t="n"/>
-      <c r="E43" s="23" t="n"/>
-      <c r="F43" s="23" t="n"/>
-      <c r="G43" s="23" t="n"/>
+      <c r="B43" s="49" t="n"/>
+      <c r="C43" s="49" t="n"/>
+      <c r="D43" s="49" t="n"/>
+      <c r="E43" s="49" t="n"/>
+      <c r="F43" s="49" t="n"/>
+      <c r="G43" s="49" t="n"/>
       <c r="H43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n"/>
-      <c r="B44" s="24" t="n"/>
-      <c r="C44" s="25" t="n"/>
-      <c r="D44" s="18" t="n"/>
-      <c r="E44" s="18" t="n"/>
-      <c r="F44" s="18" t="n"/>
-      <c r="G44" s="18" t="n"/>
+      <c r="B44" s="23" t="n"/>
+      <c r="C44" s="23" t="n"/>
+      <c r="D44" s="23" t="n"/>
+      <c r="E44" s="23" t="n"/>
+      <c r="F44" s="23" t="n"/>
+      <c r="G44" s="23" t="n"/>
       <c r="H44" s="4" t="n"/>
     </row>
     <row r="45">
+      <c r="A45" s="4" t="n"/>
       <c r="B45" s="24" t="n"/>
       <c r="C45" s="25" t="n"/>
       <c r="D45" s="18" t="n"/>
       <c r="E45" s="18" t="n"/>
       <c r="F45" s="18" t="n"/>
       <c r="G45" s="18" t="n"/>
+      <c r="H45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="24" t="n"/>
+      <c r="C46" s="25" t="n"/>
+      <c r="D46" s="18" t="n"/>
+      <c r="E46" s="18" t="n"/>
+      <c r="F46" s="18" t="n"/>
+      <c r="G46" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B34:G34"/>
+    <mergeCell ref="B35:G35"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" scale="87" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="85"/>
 </worksheet>
 </file>
</xml_diff>